<commit_message>
Added preferences model, controller, and routes + minor fixes
</commit_message>
<xml_diff>
--- a/backend-logic/data/data.xlsx
+++ b/backend-logic/data/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohammed\PlanMyMorocco\backend-logic\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mohammed\OneDrive\Database Plan My Morocco real\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4603193-9316-4319-A289-F6A3998C1869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB31EFA1-FBF6-4480-968D-C6A30308105B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{0677A140-6DE2-4459-A79C-7541D9377EF4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{0677A140-6DE2-4459-A79C-7541D9377EF4}"/>
   </bookViews>
   <sheets>
     <sheet name="Cities" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="213">
   <si>
     <t>Souk Semmarine</t>
   </si>
@@ -768,6 +768,9 @@
   </si>
   <si>
     <t>https://images.contentstack.io/v3/assets/blt06f605a34f1194ff/blt8c7da5f579a86057/6792a968bf5204e2067d25c6/iStock-1440978662-HEADERDESKTOP.jpg?format=webp&amp;auto=avif&amp;quality=60&amp;crop=16%3A9&amp;width=1440</t>
+  </si>
+  <si>
+    <t>solo</t>
   </si>
 </sst>
 </file>
@@ -1899,6 +1902,9 @@
       <c r="J2" t="s">
         <v>5</v>
       </c>
+      <c r="K2" t="s">
+        <v>212</v>
+      </c>
       <c r="L2">
         <v>0</v>
       </c>
@@ -1928,6 +1934,9 @@
       <c r="J3" t="s">
         <v>22</v>
       </c>
+      <c r="K3" t="s">
+        <v>212</v>
+      </c>
       <c r="L3">
         <v>0</v>
       </c>
@@ -1957,7 +1966,9 @@
       <c r="J4" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" t="s">
+        <v>212</v>
+      </c>
       <c r="L4">
         <v>0</v>
       </c>
@@ -1987,7 +1998,9 @@
       <c r="J5" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="K5" s="2"/>
+      <c r="K5" t="s">
+        <v>212</v>
+      </c>
       <c r="L5">
         <v>0</v>
       </c>
@@ -2017,7 +2030,9 @@
       <c r="J6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" t="s">
+        <v>212</v>
+      </c>
       <c r="L6">
         <v>0</v>
       </c>
@@ -2047,6 +2062,9 @@
       <c r="J7" t="s">
         <v>11</v>
       </c>
+      <c r="K7" t="s">
+        <v>212</v>
+      </c>
       <c r="L7">
         <v>0</v>
       </c>
@@ -2076,6 +2094,9 @@
       <c r="J8" t="s">
         <v>80</v>
       </c>
+      <c r="K8" t="s">
+        <v>212</v>
+      </c>
       <c r="L8">
         <v>0</v>
       </c>
@@ -2105,7 +2126,9 @@
       <c r="J9" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="K9" s="2"/>
+      <c r="K9" t="s">
+        <v>212</v>
+      </c>
       <c r="L9" s="3">
         <v>3.8</v>
       </c>
@@ -2135,6 +2158,9 @@
       <c r="J10" t="s">
         <v>97</v>
       </c>
+      <c r="K10" t="s">
+        <v>212</v>
+      </c>
       <c r="L10" s="3">
         <v>3.9</v>
       </c>
@@ -2164,6 +2190,9 @@
       <c r="J11" t="s">
         <v>99</v>
       </c>
+      <c r="K11" t="s">
+        <v>212</v>
+      </c>
       <c r="L11" s="3">
         <v>2.1</v>
       </c>
@@ -2193,6 +2222,9 @@
       <c r="J12" t="s">
         <v>133</v>
       </c>
+      <c r="K12" t="s">
+        <v>212</v>
+      </c>
       <c r="L12">
         <v>3</v>
       </c>
@@ -2222,6 +2254,9 @@
       <c r="J13" t="s">
         <v>1</v>
       </c>
+      <c r="K13" t="s">
+        <v>212</v>
+      </c>
       <c r="L13">
         <v>0</v>
       </c>
@@ -2251,6 +2286,9 @@
       <c r="J14" t="s">
         <v>3</v>
       </c>
+      <c r="K14" t="s">
+        <v>212</v>
+      </c>
       <c r="L14">
         <v>0</v>
       </c>
@@ -2280,7 +2318,9 @@
       <c r="J15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="2"/>
+      <c r="K15" t="s">
+        <v>212</v>
+      </c>
       <c r="L15">
         <v>0</v>
       </c>
@@ -2310,6 +2350,9 @@
       <c r="J16" t="s">
         <v>42</v>
       </c>
+      <c r="K16" t="s">
+        <v>212</v>
+      </c>
       <c r="L16">
         <v>0</v>
       </c>
@@ -2340,6 +2383,9 @@
       <c r="J17" t="s">
         <v>29</v>
       </c>
+      <c r="K17" t="s">
+        <v>212</v>
+      </c>
       <c r="L17">
         <v>0</v>
       </c>
@@ -2366,7 +2412,9 @@
       <c r="J18" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="K18" s="2"/>
+      <c r="K18" t="s">
+        <v>212</v>
+      </c>
       <c r="L18" s="3">
         <v>4.5</v>
       </c>
@@ -2396,7 +2444,9 @@
       <c r="J19" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="K19" s="2"/>
+      <c r="K19" t="s">
+        <v>212</v>
+      </c>
       <c r="L19" s="4">
         <v>4.3</v>
       </c>
@@ -2426,7 +2476,9 @@
       <c r="J20" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="K20" s="2"/>
+      <c r="K20" t="s">
+        <v>212</v>
+      </c>
       <c r="L20" s="5">
         <v>3</v>
       </c>
@@ -2456,6 +2508,9 @@
       <c r="J21" t="s">
         <v>125</v>
       </c>
+      <c r="K21" t="s">
+        <v>212</v>
+      </c>
       <c r="L21">
         <v>3.5</v>
       </c>
@@ -2485,6 +2540,9 @@
       <c r="J22" t="s">
         <v>127</v>
       </c>
+      <c r="K22" t="s">
+        <v>212</v>
+      </c>
       <c r="L22">
         <v>4</v>
       </c>
@@ -2514,6 +2572,9 @@
       <c r="J23" t="s">
         <v>130</v>
       </c>
+      <c r="K23" t="s">
+        <v>212</v>
+      </c>
       <c r="L23">
         <v>2</v>
       </c>
@@ -2543,6 +2604,9 @@
       <c r="J24" t="s">
         <v>33</v>
       </c>
+      <c r="K24" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="25" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -2572,6 +2636,9 @@
       <c r="J25" t="s">
         <v>40</v>
       </c>
+      <c r="K25" t="s">
+        <v>212</v>
+      </c>
       <c r="L25">
         <v>0</v>
       </c>
@@ -2601,7 +2668,9 @@
       <c r="J26" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="K26" s="2"/>
+      <c r="K26" t="s">
+        <v>212</v>
+      </c>
       <c r="L26">
         <v>4</v>
       </c>

</xml_diff>